<commit_message>
Sprint 1 architecture baseline and Page Inventory
</commit_message>
<xml_diff>
--- a/Documentation/Pages.xlsx
+++ b/Documentation/Pages.xlsx
@@ -8,15 +8,18 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repositories\BMMS-Legacy\Documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0804CE24-340B-448F-87A1-350CA91DAAA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BA7F84C-1FEC-4D73-AA78-4BA49D25D71C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Pages" sheetId="1" r:id="rId1"/>
     <sheet name="Reports" sheetId="2" r:id="rId2"/>
     <sheet name="DatabaseTables" sheetId="3" r:id="rId3"/>
-    <sheet name="StoredProcedures" sheetId="4" r:id="rId4"/>
+    <sheet name="DependencyInventory" sheetId="5" r:id="rId4"/>
+    <sheet name="StoredProcedures" sheetId="4" r:id="rId5"/>
+    <sheet name="Issue" sheetId="6" r:id="rId6"/>
+    <sheet name="RoleMatrix" sheetId="7" r:id="rId7"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -28,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="306" uniqueCount="229">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="350" uniqueCount="264">
   <si>
     <t>Sno</t>
   </si>
@@ -715,19 +718,130 @@
   </si>
   <si>
     <t>spr_UpdateSubjectNoByAgendaId</t>
+  </si>
+  <si>
+    <t>Component</t>
+  </si>
+  <si>
+    <t>Version</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>AjaxControlToolkit</t>
+  </si>
+  <si>
+    <t>FreeTextBox</t>
+  </si>
+  <si>
+    <t>iTextSharp</t>
+  </si>
+  <si>
+    <t>Microsoft.SqlServer.Replication</t>
+  </si>
+  <si>
+    <t>Microsoft.SqlServer.BatchParser</t>
+  </si>
+  <si>
+    <t>Microsoft Office Interop</t>
+  </si>
+  <si>
+    <t>Replace SQL Server SMO dependency</t>
+  </si>
+  <si>
+    <t>Backup Database</t>
+  </si>
+  <si>
+    <t>Reset Database</t>
+  </si>
+  <si>
+    <t>BMMS</t>
+  </si>
+  <si>
+    <t>FreeTextBox.DLL</t>
+  </si>
+  <si>
+    <t>DLL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">References   </t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>sno</t>
+  </si>
+  <si>
+    <t>Inventory</t>
+  </si>
+  <si>
+    <t>Minutes Entry</t>
+  </si>
+  <si>
+    <t>TinyMCE</t>
+  </si>
+  <si>
+    <t>CKEditor</t>
+  </si>
+  <si>
+    <t>AjaxControlToolKit</t>
+  </si>
+  <si>
+    <t>CalendarExtender</t>
+  </si>
+  <si>
+    <t>ModalPopupExtender</t>
+  </si>
+  <si>
+    <t>Validator controls</t>
+  </si>
+  <si>
+    <t>admin</t>
+  </si>
+  <si>
+    <t>Controller</t>
+  </si>
+  <si>
+    <t>secuser</t>
+  </si>
+  <si>
+    <t>Manager</t>
+  </si>
+  <si>
+    <t>credmanager</t>
+  </si>
+  <si>
+    <t>creduser</t>
+  </si>
+  <si>
+    <t>Username</t>
+  </si>
+  <si>
+    <t>LoginName</t>
+  </si>
+  <si>
+    <t>Roleid</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color theme="1"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -750,8 +864,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1874,6 +1991,82 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{47EDB5EC-739B-4F6D-BE77-90C272B76917}">
+  <dimension ref="A1:D7"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="21.6640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>229</v>
+      </c>
+      <c r="C1" t="s">
+        <v>230</v>
+      </c>
+      <c r="D1" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>237</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FAC2B4CE-15A2-4381-8BE9-775FECE206F7}">
   <dimension ref="A1:B141"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -3012,4 +3205,194 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1CC44D31-C505-408D-97AB-57B4DA0CE83F}">
+  <dimension ref="A1:F9"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="31.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.88671875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="21" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>246</v>
+      </c>
+      <c r="B1" t="s">
+        <v>245</v>
+      </c>
+      <c r="C1" t="s">
+        <v>247</v>
+      </c>
+      <c r="D1" t="s">
+        <v>243</v>
+      </c>
+      <c r="E1" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>238</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C3" s="1" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>2</v>
+      </c>
+      <c r="B4" t="s">
+        <v>233</v>
+      </c>
+      <c r="C4" t="s">
+        <v>241</v>
+      </c>
+      <c r="D4" t="s">
+        <v>242</v>
+      </c>
+      <c r="E4" t="s">
+        <v>233</v>
+      </c>
+      <c r="F4" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C5" t="s">
+        <v>32</v>
+      </c>
+      <c r="F5" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C6" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>3</v>
+      </c>
+      <c r="B7" t="s">
+        <v>251</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>252</v>
+      </c>
+      <c r="D7" t="s">
+        <v>251</v>
+      </c>
+      <c r="E7" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C8" s="1" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C9" s="1" t="s">
+        <v>254</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E0B494A3-FD67-496E-BA42-E576CA0F9B6A}">
+  <dimension ref="B1:E5"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" t="s">
+        <v>261</v>
+      </c>
+      <c r="D1" t="s">
+        <v>262</v>
+      </c>
+      <c r="E1" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="2" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s">
+        <v>255</v>
+      </c>
+      <c r="D2" t="s">
+        <v>255</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B3">
+        <v>2</v>
+      </c>
+      <c r="C3" t="s">
+        <v>256</v>
+      </c>
+      <c r="D3" t="s">
+        <v>257</v>
+      </c>
+      <c r="E3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B4">
+        <v>3</v>
+      </c>
+      <c r="C4" t="s">
+        <v>258</v>
+      </c>
+      <c r="D4" t="s">
+        <v>259</v>
+      </c>
+      <c r="E4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B5">
+        <v>4</v>
+      </c>
+      <c r="C5" t="s">
+        <v>27</v>
+      </c>
+      <c r="D5" t="s">
+        <v>260</v>
+      </c>
+      <c r="E5">
+        <v>4</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>